<commit_message>
Reset experiment to base and preserve s001 stories
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/secuencia/s001/docs/DoE_VibeCoding_Sequence_s001.xlsx
+++ b/secuencia/s001/docs/DoE_VibeCoding_Sequence_s001.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>Secuencia de investigación desarrollo Vibe Coding</t>
   </si>
@@ -95,102 +95,12 @@
   <si>
     <t>Creación de la estructura base (usando CONTEXT.md de secuencia)</t>
   </si>
-  <si>
-    <t>A1</t>
-  </si>
-  <si>
-    <t>Creación de historia A1, prueba de Contexto y Project.md</t>
-  </si>
-  <si>
-    <t>A3</t>
-  </si>
-  <si>
-    <t>Completa la historia A3 Regresión Ok</t>
-  </si>
-  <si>
-    <t>Fallo PyRight</t>
-  </si>
-  <si>
-    <t>A2</t>
-  </si>
-  <si>
-    <t>C1</t>
-  </si>
-  <si>
-    <t>se agrego  UniformParameterSampler y sample_uniform_parameters() para muestrear un ModelParameters</t>
-  </si>
-  <si>
-    <t>C2</t>
-  </si>
-  <si>
-    <t>Agregué la interfaz Policy,  el motor simulate_deterministic_sprints() y la API run_monte_carlo()</t>
-  </si>
-  <si>
-    <t>MonteCarloRunResult con métricas por corrida, agregué MetricSummary y aggregate_metrics()</t>
-  </si>
-  <si>
-    <t>C3</t>
-  </si>
-  <si>
-    <t>Agregué FixedRemediationPolicy, el módulo optimization.py con GridSearchEvaluation, GridSearchResult y search_optimal_remediation_fraction()</t>
-  </si>
-  <si>
-    <t>D1</t>
-  </si>
-  <si>
-    <t>D2</t>
-  </si>
-  <si>
-    <t>D3</t>
-  </si>
-  <si>
-    <t>E1</t>
-  </si>
-  <si>
-    <t>E2</t>
-  </si>
-  <si>
-    <t>E3</t>
-  </si>
-  <si>
-    <t>F1</t>
-  </si>
-  <si>
-    <t>F2</t>
-  </si>
-  <si>
-    <t>F3</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Agregué EconomicObjectiveFunction con pesos configurables para valor entregado, penalización por deuda remanente y penalización por sprints, la integré con search_optimal_remediation_fraction() y la reutilicé para calcular total_economic_value en Monte Carlo</t>
-  </si>
-  <si>
-    <t>B1</t>
-  </si>
-  <si>
-    <t>BacklogFirstPolicy integrada a simulate_deterministic_sprints()</t>
-  </si>
-  <si>
-    <t>B2</t>
-  </si>
-  <si>
-    <t>B3</t>
-  </si>
-  <si>
-    <t>regresión explícita para ProportionalDebtPolicy integrada a simulate_deterministic_sprints(</t>
-  </si>
-  <si>
-    <t>añadí una prueba de integración parametrizada que verifica que DebtFirstPolicy, BacklogFirstPolicy y ProportionalDebtPolicy cumplen el protocolo y pueden intercambiarse en simulate_deterministic_sprints()</t>
-  </si>
-  <si>
-    <t>B4</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -209,14 +119,6 @@
     <font>
       <b/>
       <sz val="18"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -296,7 +198,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -307,8 +209,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -324,6 +224,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -638,13 +539,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:M883"/>
+  <dimension ref="B2:M877"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="17.375" customWidth="1"/>
-    <col min="4" max="4" width="14.375" customWidth="1"/>
+    <col min="3" max="3" width="11.75" bestFit="1" customWidth="1"/>
     <col min="5" max="12" width="15.875" customWidth="1"/>
-    <col min="13" max="13" width="103.375" customWidth="1"/>
+    <col min="13" max="13" width="57.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:13" ht="23.25" x14ac:dyDescent="0.35">
@@ -666,7 +566,7 @@
       <c r="B6" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="13">
         <f>DATE(2026,5,20)</f>
         <v>46162</v>
       </c>
@@ -683,46 +583,46 @@
       <c r="B8" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="C8" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="14"/>
-      <c r="J8" s="14"/>
-      <c r="K8" s="14"/>
-      <c r="L8" s="14"/>
-      <c r="M8" s="14"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="12"/>
+      <c r="F8" s="12"/>
+      <c r="G8" s="12"/>
+      <c r="H8" s="12"/>
+      <c r="I8" s="12"/>
+      <c r="J8" s="12"/>
+      <c r="K8" s="12"/>
+      <c r="L8" s="12"/>
+      <c r="M8" s="12"/>
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="C10" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="E10" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="F10" s="10"/>
-      <c r="G10" s="10"/>
-      <c r="H10" s="10"/>
-      <c r="I10" s="10"/>
-      <c r="J10" s="10"/>
-      <c r="K10" s="10"/>
-      <c r="L10" s="10"/>
-      <c r="M10" s="10"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
+      <c r="K10" s="8"/>
+      <c r="L10" s="8"/>
+      <c r="M10" s="8"/>
     </row>
     <row r="11" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B11" s="11"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="11"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="9"/>
       <c r="E11" s="4" t="s">
         <v>7</v>
       </c>
@@ -790,53 +690,23 @@
       </c>
     </row>
     <row r="13" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B13" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C13" s="2">
-        <v>13</v>
-      </c>
-      <c r="D13" s="2">
-        <v>0</v>
-      </c>
-      <c r="E13" s="2">
-        <v>0</v>
-      </c>
-      <c r="F13" s="2">
-        <v>0</v>
-      </c>
-      <c r="G13" s="2">
-        <v>0</v>
-      </c>
-      <c r="H13" s="2">
-        <v>0</v>
-      </c>
-      <c r="I13" s="2">
-        <v>0</v>
-      </c>
-      <c r="J13" s="2">
-        <v>0</v>
-      </c>
-      <c r="K13" s="2">
-        <v>0</v>
-      </c>
-      <c r="L13" s="2">
-        <v>0</v>
-      </c>
-      <c r="M13" s="2" t="s">
-        <v>21</v>
-      </c>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2"/>
+      <c r="L13" s="2"/>
+      <c r="M13" s="2"/>
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B14" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C14" s="2">
-        <v>14</v>
-      </c>
-      <c r="D14" s="2">
-        <v>0</v>
-      </c>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
@@ -848,52 +718,32 @@
       <c r="M14" s="2"/>
     </row>
     <row r="15" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B15" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C15" s="2">
-        <v>19</v>
-      </c>
-      <c r="D15" s="2">
-        <v>1</v>
-      </c>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
-      <c r="I15" s="2">
-        <v>1</v>
-      </c>
+      <c r="I15" s="2"/>
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
       <c r="L15" s="2"/>
-      <c r="M15" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="M15" s="2"/>
     </row>
     <row r="16" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B16" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C16" s="2">
-        <v>15</v>
-      </c>
-      <c r="D16" s="2">
-        <v>2</v>
-      </c>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
-      <c r="K16" s="2">
-        <v>0</v>
-      </c>
+      <c r="K16" s="2"/>
       <c r="L16" s="2"/>
-      <c r="M16" s="2" t="s">
-        <v>23</v>
-      </c>
+      <c r="M16" s="2"/>
     </row>
     <row r="17" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B17" s="2"/>
@@ -910,154 +760,60 @@
       <c r="M17" s="2"/>
     </row>
     <row r="18" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B18" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C18" s="2">
-        <v>15</v>
-      </c>
-      <c r="D18" s="2">
-        <v>0</v>
-      </c>
-      <c r="E18" s="2">
-        <v>0</v>
-      </c>
-      <c r="F18" s="2">
-        <v>0</v>
-      </c>
-      <c r="G18" s="2">
-        <v>0</v>
-      </c>
-      <c r="H18" s="2">
-        <v>0</v>
-      </c>
-      <c r="I18" s="2">
-        <v>0</v>
-      </c>
-      <c r="J18" s="2">
-        <v>0</v>
-      </c>
-      <c r="K18" s="2">
-        <v>0</v>
-      </c>
-      <c r="L18" s="2">
-        <v>0</v>
-      </c>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="2"/>
+      <c r="K18" s="2"/>
+      <c r="L18" s="2"/>
       <c r="M18" s="2"/>
     </row>
     <row r="19" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B19" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C19" s="2">
-        <v>17</v>
-      </c>
-      <c r="D19" s="2">
-        <v>0</v>
-      </c>
-      <c r="E19" s="2">
-        <v>0</v>
-      </c>
-      <c r="F19" s="2">
-        <v>0</v>
-      </c>
-      <c r="G19" s="2">
-        <v>0</v>
-      </c>
-      <c r="H19" s="2">
-        <v>0</v>
-      </c>
-      <c r="I19" s="2">
-        <v>0</v>
-      </c>
-      <c r="J19" s="2">
-        <v>0</v>
-      </c>
-      <c r="K19" s="2">
-        <v>0</v>
-      </c>
-      <c r="L19" s="2">
-        <v>0</v>
-      </c>
-      <c r="M19" s="2" t="s">
-        <v>44</v>
-      </c>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+      <c r="J19" s="2"/>
+      <c r="K19" s="2"/>
+      <c r="L19" s="2"/>
+      <c r="M19" s="2"/>
     </row>
     <row r="20" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B20" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C20" s="2">
-        <v>16</v>
-      </c>
-      <c r="D20" s="2">
-        <v>0</v>
-      </c>
-      <c r="E20" s="2">
-        <v>0</v>
-      </c>
-      <c r="F20" s="2">
-        <v>0</v>
-      </c>
-      <c r="G20" s="2">
-        <v>0</v>
-      </c>
-      <c r="H20" s="2">
-        <v>0</v>
-      </c>
-      <c r="I20" s="2">
-        <v>0</v>
-      </c>
-      <c r="J20" s="2">
-        <v>0</v>
-      </c>
-      <c r="K20" s="2">
-        <v>0</v>
-      </c>
-      <c r="L20" s="2">
-        <v>0</v>
-      </c>
-      <c r="M20" s="2" t="s">
-        <v>47</v>
-      </c>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
+      <c r="J20" s="2"/>
+      <c r="K20" s="2"/>
+      <c r="L20" s="2"/>
+      <c r="M20" s="2"/>
     </row>
     <row r="21" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B21" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C21" s="2">
-        <v>12</v>
-      </c>
-      <c r="D21" s="2">
-        <v>0</v>
-      </c>
-      <c r="E21" s="2">
-        <v>0</v>
-      </c>
-      <c r="F21" s="2">
-        <v>0</v>
-      </c>
-      <c r="G21" s="2">
-        <v>0</v>
-      </c>
-      <c r="H21" s="2">
-        <v>0</v>
-      </c>
-      <c r="I21" s="2">
-        <v>0</v>
-      </c>
-      <c r="J21" s="2">
-        <v>0</v>
-      </c>
-      <c r="K21" s="2">
-        <v>0</v>
-      </c>
-      <c r="L21" s="2">
-        <v>0</v>
-      </c>
-      <c r="M21" s="2" t="s">
-        <v>48</v>
-      </c>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
+      <c r="F21" s="2"/>
+      <c r="G21" s="2"/>
+      <c r="H21" s="2"/>
+      <c r="I21" s="2"/>
+      <c r="J21" s="2"/>
+      <c r="K21" s="2"/>
+      <c r="L21" s="2"/>
+      <c r="M21" s="2"/>
     </row>
     <row r="22" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B22" s="2"/>
@@ -1088,118 +844,46 @@
       <c r="M23" s="2"/>
     </row>
     <row r="24" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B24" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C24" s="2">
-        <v>32</v>
-      </c>
-      <c r="D24" s="2">
-        <v>0</v>
-      </c>
-      <c r="E24" s="2">
-        <v>0</v>
-      </c>
-      <c r="F24" s="2">
-        <v>0</v>
-      </c>
-      <c r="G24" s="2">
-        <v>0</v>
-      </c>
-      <c r="H24" s="2">
-        <v>0</v>
-      </c>
-      <c r="I24" s="2">
-        <v>0</v>
-      </c>
-      <c r="J24" s="2">
-        <v>0</v>
-      </c>
-      <c r="K24" s="2">
-        <v>0</v>
-      </c>
-      <c r="L24" s="2">
-        <v>0</v>
-      </c>
-      <c r="M24" s="2" t="s">
-        <v>27</v>
-      </c>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="2"/>
+      <c r="K24" s="2"/>
+      <c r="L24" s="2"/>
+      <c r="M24" s="2"/>
     </row>
     <row r="25" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B25" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C25" s="2">
-        <v>34</v>
-      </c>
-      <c r="D25" s="2">
-        <v>0</v>
-      </c>
-      <c r="E25" s="2">
-        <v>0</v>
-      </c>
-      <c r="F25" s="2">
-        <v>0</v>
-      </c>
-      <c r="G25" s="2">
-        <v>0</v>
-      </c>
-      <c r="H25" s="2">
-        <v>0</v>
-      </c>
-      <c r="I25" s="2">
-        <v>0</v>
-      </c>
-      <c r="J25" s="2">
-        <v>0</v>
-      </c>
-      <c r="K25" s="2">
-        <v>0</v>
-      </c>
-      <c r="L25" s="2">
-        <v>0</v>
-      </c>
-      <c r="M25" s="2" t="s">
-        <v>29</v>
-      </c>
+      <c r="B25" s="2"/>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+      <c r="E25" s="2"/>
+      <c r="F25" s="2"/>
+      <c r="G25" s="2"/>
+      <c r="H25" s="2"/>
+      <c r="I25" s="2"/>
+      <c r="J25" s="2"/>
+      <c r="K25" s="2"/>
+      <c r="L25" s="2"/>
+      <c r="M25" s="2"/>
     </row>
     <row r="26" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B26" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C26" s="2">
-        <v>38</v>
-      </c>
-      <c r="D26" s="2">
-        <v>0</v>
-      </c>
-      <c r="E26" s="2">
-        <v>0</v>
-      </c>
-      <c r="F26" s="2">
-        <v>0</v>
-      </c>
-      <c r="G26" s="2">
-        <v>0</v>
-      </c>
-      <c r="H26" s="2">
-        <v>0</v>
-      </c>
-      <c r="I26" s="2">
-        <v>0</v>
-      </c>
-      <c r="J26" s="2">
-        <v>0</v>
-      </c>
-      <c r="K26" s="2">
-        <v>0</v>
-      </c>
-      <c r="L26" s="2">
-        <v>0</v>
-      </c>
-      <c r="M26" s="2" t="s">
-        <v>30</v>
-      </c>
+      <c r="B26" s="2"/>
+      <c r="C26" s="2"/>
+      <c r="D26" s="2"/>
+      <c r="E26" s="2"/>
+      <c r="F26" s="2"/>
+      <c r="G26" s="2"/>
+      <c r="H26" s="2"/>
+      <c r="I26" s="2"/>
+      <c r="J26" s="2"/>
+      <c r="K26" s="2"/>
+      <c r="L26" s="2"/>
+      <c r="M26" s="2"/>
     </row>
     <row r="27" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B27" s="2"/>
@@ -1216,32 +900,22 @@
       <c r="M27" s="2"/>
     </row>
     <row r="28" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B28" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C28" s="2">
-        <v>44</v>
-      </c>
+      <c r="B28" s="2"/>
+      <c r="C28" s="2"/>
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
       <c r="I28" s="2"/>
-      <c r="J28" s="9"/>
+      <c r="J28" s="2"/>
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
-      <c r="M28" s="2" t="s">
-        <v>32</v>
-      </c>
+      <c r="M28" s="2"/>
     </row>
     <row r="29" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B29" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C29" s="2">
-        <v>31</v>
-      </c>
+      <c r="B29" s="2"/>
+      <c r="C29" s="2"/>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
       <c r="F29" s="2"/>
@@ -1251,14 +925,10 @@
       <c r="J29" s="2"/>
       <c r="K29" s="2"/>
       <c r="L29" s="2"/>
-      <c r="M29" s="2" t="s">
-        <v>42</v>
-      </c>
+      <c r="M29" s="2"/>
     </row>
     <row r="30" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B30" s="2" t="s">
-        <v>35</v>
-      </c>
+      <c r="B30" s="2"/>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
@@ -1286,9 +956,7 @@
       <c r="M31" s="2"/>
     </row>
     <row r="32" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B32" s="2" t="s">
-        <v>36</v>
-      </c>
+      <c r="B32" s="2"/>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
       <c r="E32" s="2"/>
@@ -1302,9 +970,7 @@
       <c r="M32" s="2"/>
     </row>
     <row r="33" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B33" s="2" t="s">
-        <v>37</v>
-      </c>
+      <c r="B33" s="2"/>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
       <c r="E33" s="2"/>
@@ -1318,9 +984,7 @@
       <c r="M33" s="2"/>
     </row>
     <row r="34" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B34" s="2" t="s">
-        <v>38</v>
-      </c>
+      <c r="B34" s="2"/>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
       <c r="E34" s="2"/>
@@ -1348,9 +1012,7 @@
       <c r="M35" s="2"/>
     </row>
     <row r="36" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B36" s="2" t="s">
-        <v>39</v>
-      </c>
+      <c r="B36" s="2"/>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
       <c r="E36" s="2"/>
@@ -1364,9 +1026,7 @@
       <c r="M36" s="2"/>
     </row>
     <row r="37" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B37" s="2" t="s">
-        <v>40</v>
-      </c>
+      <c r="B37" s="2"/>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
       <c r="E37" s="2"/>
@@ -1380,9 +1040,7 @@
       <c r="M37" s="2"/>
     </row>
     <row r="38" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B38" s="2" t="s">
-        <v>41</v>
-      </c>
+      <c r="B38" s="2"/>
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
       <c r="E38" s="2"/>
@@ -13141,90 +12799,6 @@
       <c r="L877" s="2"/>
       <c r="M877" s="2"/>
     </row>
-    <row r="878" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B878" s="2"/>
-      <c r="C878" s="2"/>
-      <c r="D878" s="2"/>
-      <c r="E878" s="2"/>
-      <c r="F878" s="2"/>
-      <c r="G878" s="2"/>
-      <c r="H878" s="2"/>
-      <c r="I878" s="2"/>
-      <c r="J878" s="2"/>
-      <c r="K878" s="2"/>
-      <c r="L878" s="2"/>
-      <c r="M878" s="2"/>
-    </row>
-    <row r="879" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B879" s="2"/>
-      <c r="C879" s="2"/>
-      <c r="D879" s="2"/>
-      <c r="E879" s="2"/>
-      <c r="F879" s="2"/>
-      <c r="G879" s="2"/>
-      <c r="H879" s="2"/>
-      <c r="I879" s="2"/>
-      <c r="J879" s="2"/>
-      <c r="K879" s="2"/>
-      <c r="L879" s="2"/>
-      <c r="M879" s="2"/>
-    </row>
-    <row r="880" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B880" s="2"/>
-      <c r="C880" s="2"/>
-      <c r="D880" s="2"/>
-      <c r="E880" s="2"/>
-      <c r="F880" s="2"/>
-      <c r="G880" s="2"/>
-      <c r="H880" s="2"/>
-      <c r="I880" s="2"/>
-      <c r="J880" s="2"/>
-      <c r="K880" s="2"/>
-      <c r="L880" s="2"/>
-      <c r="M880" s="2"/>
-    </row>
-    <row r="881" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B881" s="2"/>
-      <c r="C881" s="2"/>
-      <c r="D881" s="2"/>
-      <c r="E881" s="2"/>
-      <c r="F881" s="2"/>
-      <c r="G881" s="2"/>
-      <c r="H881" s="2"/>
-      <c r="I881" s="2"/>
-      <c r="J881" s="2"/>
-      <c r="K881" s="2"/>
-      <c r="L881" s="2"/>
-      <c r="M881" s="2"/>
-    </row>
-    <row r="882" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B882" s="2"/>
-      <c r="C882" s="2"/>
-      <c r="D882" s="2"/>
-      <c r="E882" s="2"/>
-      <c r="F882" s="2"/>
-      <c r="G882" s="2"/>
-      <c r="H882" s="2"/>
-      <c r="I882" s="2"/>
-      <c r="J882" s="2"/>
-      <c r="K882" s="2"/>
-      <c r="L882" s="2"/>
-      <c r="M882" s="2"/>
-    </row>
-    <row r="883" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B883" s="2"/>
-      <c r="C883" s="2"/>
-      <c r="D883" s="2"/>
-      <c r="E883" s="2"/>
-      <c r="F883" s="2"/>
-      <c r="G883" s="2"/>
-      <c r="H883" s="2"/>
-      <c r="I883" s="2"/>
-      <c r="J883" s="2"/>
-      <c r="K883" s="2"/>
-      <c r="L883" s="2"/>
-      <c r="M883" s="2"/>
-    </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="E10:M10"/>

</xml_diff>